<commit_message>
Fix Task Scheduler action parameters and update publishing schedule with Day 2 9AM short
</commit_message>
<xml_diff>
--- a/data/publishing_schedule.xlsx
+++ b/data/publishing_schedule.xlsx
@@ -717,10 +717,14 @@
           <t>A business is worth the present value of its future cash flows; see what the discount rate does.</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Most investors don't realize that a company is actually worth just the present value of its future cash flows. Money tomorrow is worth less than money today. We use a discount rate to shrink future earnings down into today's actual value. If you apply a higher discount rate, perceived risk shoots up, drastically reducing the total calculated valuation of the entire business. When RBI interest rates shift across India, the discount rate changes, d</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -761,10 +765,14 @@
           <t>Read P/E as the inverse of earnings yield and compare it with bond yields.</t>
         </is>
       </c>
-      <c r="I5" s="10" t="inlineStr"/>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>Most investors don't realize that the classic price-to-earnings ratio is actually just the inverse of your earnings yield. If a company trades at a P/E of twenty, its earnings yield is five percent, calculated by dividing one by twenty. You must compare this stock earnings yield directly against risk-free bond yields to see if equities are genuinely attractive. In the Indian markets, when NSE stock P/E ratios soar high, earnings yields drop below</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(storage): add state store, atomic persistence, and Excel reconciliation (#20, #12)
</commit_message>
<xml_diff>
--- a/data/publishing_schedule.xlsx
+++ b/data/publishing_schedule.xlsx
@@ -2449,6 +2449,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="J2:J43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Done,Pending,In progress,Failed"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(schedule): reset D04-09:00 to Pending for seamless upcoming publication
</commit_message>
<xml_diff>
--- a/data/publishing_schedule.xlsx
+++ b/data/publishing_schedule.xlsx
@@ -1068,9 +1068,9 @@
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr"/>
-      <c r="J11" s="13" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>